<commit_message>
Initial Commit Have it reading from the Excel File now.
</commit_message>
<xml_diff>
--- a/Fleet_Equipment_Database.xlsx
+++ b/Fleet_Equipment_Database.xlsx
@@ -427,40 +427,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="n">
-        <v>3</v>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Parameter_Header</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Peterbilt_579_UltraLoft</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Volvo_VNL_860</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Kenworth_T680_NextGen</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Ford_F450_Pickup</t>
+        </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Chassis_Key</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Peterbilt_579_UltraLoft</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Volvo_VNL_860</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Kenworth_T680_NextGen</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Ford_F450_Pickup</t>
         </is>
@@ -469,20 +487,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Manufacturer</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Peterbilt</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Volvo</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Kenworth</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Ford</t>
         </is>
@@ -491,84 +514,111 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Model_Designation</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>579 UltraLoft</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>VNL 860</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>T680 Next Gen</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>F-450 Super Duty (DRW Crew Cab)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Base_Tractor_Weight_lbs</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>18200</v>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
         <v>18900</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>18400</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>8600</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Drag_Coefficient_Cd</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>0.46</v>
       </c>
-      <c r="B6" t="n">
+      <c r="C6" t="n">
         <v>0.43</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>0.45</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>0.41</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Frontal_Area_SqFt</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>104</v>
       </c>
-      <c r="B7" t="n">
+      <c r="C7" t="n">
         <v>102</v>
       </c>
-      <c r="C7" t="n">
+      <c r="D7" t="n">
         <v>103</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>48</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Aero_Constant_CdA</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>47.84</v>
       </c>
-      <c r="B8" t="n">
+      <c r="C8" t="n">
         <v>43.86</v>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>46.35</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>19.68</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>53000</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Max_Chassis_GVWR_lbs</t>
+        </is>
       </c>
       <c r="B9" t="n">
         <v>53000</v>
@@ -577,74 +627,238 @@
         <v>53000</v>
       </c>
       <c r="D9" t="n">
+        <v>53000</v>
+      </c>
+      <c r="E9" t="n">
         <v>14000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Cummins_X15_Eff, Cummins_X15_Perf</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Volvo_D13TC</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Cummins_X15_Eff, Cummins_X15_Perf</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Ford_67L_Powerstroke_HO</t>
-        </is>
+          <t>Max_Chassis_GCWR_lbs</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>80000</v>
+      </c>
+      <c r="C10" t="n">
+        <v>80000</v>
+      </c>
+      <c r="D10" t="n">
+        <v>80000</v>
+      </c>
+      <c r="E10" t="n">
+        <v>35000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Eaton_Endurant_12</t>
+          <t>Valid_Engines_List</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Volvo_IShift_Direct, Volvo_IShift_OD</t>
+          <t>Cummins_X15_Eff, Cummins_X15_Perf</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Eaton_Endurant_12</t>
+          <t>Volvo_D13TC</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Ford_TorqShift_10R140</t>
+          <t>Cummins_X15_Eff, Cummins_X15_Perf</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Ford_67L_Powerstroke_HO</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2.47, 2.64, 2.79, 2.93, 3.08, 3.25, 3.42</t>
+          <t>Valid_Transmissions_List</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2.15, 2.28, 2.47, 2.64, 2.85, 2.93, 3.08</t>
+          <t>Eaton_Endurant_12</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.47, 2.64, 2.79, 2.93, 3.08, 3.25, 3.42</t>
+          <t>Volvo_IShift_Direct, Volvo_IShift_OD</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>4.3</t>
-        </is>
-      </c>
+          <t>Eaton_Endurant_12</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Ford_TorqShift_10R140</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Rear_Axle_Ratio_1</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="C13" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="E13" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Rear_Axle_Ratio_2</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="C14" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Rear_Axle_Ratio_3</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="C15" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="E15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Rear_Axle_Ratio_4</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Rear_Axle_Ratio_5</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="E17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Rear_Axle_Ratio_6</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="C18" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Rear_Axle_Ratio_7</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="C19" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Rear_Axle_Ratio_8</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Rear_Axle_Ratio_9</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Rear_Axle_Ratio_10</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -657,40 +871,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="n">
-        <v>3</v>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Parameter_Header</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Cummins_X15_Eff</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Cummins_X15_Perf</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Volvo_D13TC</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Ford_67L_Powerstroke_HO</t>
+        </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Engine_Key</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Cummins_X15_Eff</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Cummins_X15_Perf</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Volvo_D13TC</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Ford_67L_Powerstroke_HO</t>
         </is>
@@ -699,20 +931,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>MANUFACTURER</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Cummins</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Cummins</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Volvo</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Ford (Super Duty Powertrains)</t>
         </is>
@@ -721,176 +958,233 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>ENGINE_FAMILY</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>X15 Efficiency (450 ST2)</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>X15 Performance (605)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>D13 Turbo Compound (455TC)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>6.7L High Output Powerstroke V8</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>14.9</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DISPLACEMENT_LITERS</t>
+        </is>
       </c>
       <c r="B5" t="n">
         <v>14.9</v>
       </c>
       <c r="C5" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="D5" t="n">
         <v>12.8</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>6.7</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PEAK_HP</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>450</v>
       </c>
-      <c r="B6" t="n">
+      <c r="C6" t="n">
         <v>605</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>455</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>500</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PEAK_HP_RPM</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>1600</v>
       </c>
-      <c r="B7" t="n">
+      <c r="C7" t="n">
         <v>1700</v>
       </c>
-      <c r="C7" t="n">
+      <c r="D7" t="n">
         <v>1400</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>2600</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>TORQUE_PROFILE_TYPE</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>Multi-Torque</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Fixed Torque</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Multi-Torque</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Fixed Torque Curve</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TORQUE_BASE_LBFT</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>1550</v>
       </c>
-      <c r="B9" t="n">
+      <c r="C9" t="n">
         <v>2050</v>
       </c>
-      <c r="C9" t="n">
+      <c r="D9" t="n">
         <v>1750</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TORQUE_TOP_LBFT</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>1750</v>
       </c>
-      <c r="B10" t="n">
+      <c r="C10" t="n">
         <v>2050</v>
       </c>
-      <c r="C10" t="n">
+      <c r="D10" t="n">
         <v>1850</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>FLAT_TORQUE_START_RPM</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>950</v>
       </c>
-      <c r="B11" t="n">
+      <c r="C11" t="n">
         <v>1000</v>
       </c>
-      <c r="C11" t="n">
+      <c r="D11" t="n">
         <v>900</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>1600</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>FLAT_TORQUE_END_RPM</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>1300</v>
       </c>
-      <c r="B12" t="n">
+      <c r="C12" t="n">
         <v>1400</v>
       </c>
-      <c r="C12" t="n">
+      <c r="D12" t="n">
         <v>1300</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>2200</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ENGINE_REDLINE_RPM</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>1900</v>
       </c>
-      <c r="B13" t="n">
+      <c r="C13" t="n">
         <v>2000</v>
       </c>
-      <c r="C13" t="n">
+      <c r="D13" t="n">
         <v>1900</v>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>4000</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>MAX_BRAKING_HP</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
         <v>450</v>
       </c>
-      <c r="B14" t="n">
+      <c r="C14" t="n">
         <v>600</v>
       </c>
-      <c r="C14" t="n">
+      <c r="D14" t="n">
         <v>530</v>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
         <v>250</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
-        <v>600</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ENGINE_IDLE_RPM</t>
+        </is>
       </c>
       <c r="B15" t="n">
         <v>600</v>
@@ -899,126 +1193,169 @@
         <v>600</v>
       </c>
       <c r="D15" t="n">
+        <v>600</v>
+      </c>
+      <c r="E15" t="n">
         <v>700</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ENGINE_IDLE_TORQUE_LBFT</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
         <v>700</v>
       </c>
-      <c r="B16" t="n">
+      <c r="C16" t="n">
         <v>800</v>
       </c>
-      <c r="C16" t="n">
+      <c r="D16" t="n">
         <v>750</v>
       </c>
-      <c r="D16" t="n">
+      <c r="E16" t="n">
         <v>450</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>LUGGING_ZONE_RISK</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>High Damage Risk</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>High Damage Risk</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Low-Speed Adaptive</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Severe Performance Drop</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BEST_BSFC_VALUE</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
         <v>0.285</v>
       </c>
-      <c r="B18" t="n">
+      <c r="C18" t="n">
         <v>0.31</v>
       </c>
-      <c r="C18" t="n">
+      <c r="D18" t="n">
         <v>0.278</v>
       </c>
-      <c r="D18" t="n">
+      <c r="E18" t="n">
         <v>0.4</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BSFC_ISLAND_LOW_RPM</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
         <v>1000</v>
       </c>
-      <c r="B19" t="n">
+      <c r="C19" t="n">
         <v>1100</v>
       </c>
-      <c r="C19" t="n">
+      <c r="D19" t="n">
         <v>950</v>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="n">
         <v>1500</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BSFC_ISLAND_HIGH_RPM</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
         <v>1250</v>
       </c>
-      <c r="B20" t="n">
+      <c r="C20" t="n">
         <v>1350</v>
       </c>
-      <c r="C20" t="n">
+      <c r="D20" t="n">
         <v>1150</v>
       </c>
-      <c r="D20" t="n">
+      <c r="E20" t="n">
         <v>2100</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BSFC_ISLAND_MIN_LOAD_PCT</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
         <v>0.45</v>
       </c>
-      <c r="B21" t="n">
+      <c r="C21" t="n">
         <v>0.5</v>
       </c>
-      <c r="C21" t="n">
+      <c r="D21" t="n">
         <v>0.4</v>
       </c>
-      <c r="D21" t="n">
+      <c r="E21" t="n">
         <v>0.35</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BSFC_ISLAND_MAX_LOAD_PCT</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
         <v>0.85</v>
       </c>
-      <c r="B22" t="n">
+      <c r="C22" t="n">
         <v>0.8</v>
       </c>
-      <c r="C22" t="n">
+      <c r="D22" t="n">
         <v>0.85</v>
       </c>
-      <c r="D22" t="n">
+      <c r="E22" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>OUTSIDE_ISLAND_PENALTY_PER_100RPM</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
         <v>0.04</v>
       </c>
-      <c r="B23" t="n">
+      <c r="C23" t="n">
         <v>0.05</v>
       </c>
-      <c r="C23" t="n">
+      <c r="D23" t="n">
         <v>0.03</v>
       </c>
-      <c r="D23" t="n">
+      <c r="E23" t="n">
         <v>0.006</v>
       </c>
     </row>
@@ -1033,40 +1370,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="n">
-        <v>3</v>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Parameter_Header</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Volvo_IShift_Direct</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Volvo_IShift_OD</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Eaton_Endurant_12</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Ford_TorqShift_10R140</t>
+        </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Transmission_Key</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Volvo_IShift_Direct</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Volvo_IShift_OD</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Eaton_Endurant_12</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Ford_TorqShift_10R140</t>
         </is>
@@ -1075,20 +1430,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Manufacturer</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Volvo</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Volvo</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Eaton Cummins</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Ford Motor Company</t>
         </is>
@@ -1097,20 +1457,25 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Model_Series</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>I-Shift AT Series</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>I-Shift ATO Series</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Endurant 12-Speed</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>TorqShift 10R140</t>
         </is>
@@ -1119,28 +1484,35 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Drivetrain_Type</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Direct Drive</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Overdrive</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Overdrive</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Overdrive</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>12</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Forward_Gears_Count</t>
+        </is>
       </c>
       <c r="B6" t="n">
         <v>12</v>
@@ -1149,214 +1521,292 @@
         <v>12</v>
       </c>
       <c r="D6" t="n">
+        <v>12</v>
+      </c>
+      <c r="E6" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>1920</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Max_Input_Torque_lbft</t>
+        </is>
       </c>
       <c r="B7" t="n">
         <v>1920</v>
       </c>
       <c r="C7" t="n">
+        <v>1920</v>
+      </c>
+      <c r="D7" t="n">
         <v>1850</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>1250</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>125000</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Max_GCW_Limit_lbs</t>
+        </is>
       </c>
       <c r="B8" t="n">
         <v>125000</v>
       </c>
       <c r="C8" t="n">
+        <v>125000</v>
+      </c>
+      <c r="D8" t="n">
         <v>110000</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>43500</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Fluid_Friction_Loss_Pct</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>0.03</v>
-      </c>
-      <c r="B9" t="n">
-        <v>0.06</v>
       </c>
       <c r="C9" t="n">
         <v>0.06</v>
       </c>
       <c r="D9" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E9" t="n">
         <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Gear_1_Ratio</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>14.94</v>
       </c>
-      <c r="B10" t="n">
+      <c r="C10" t="n">
         <v>11.73</v>
       </c>
-      <c r="C10" t="n">
+      <c r="D10" t="n">
         <v>14.43</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>4.7</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Gear_2_Ratio</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>11.73</v>
       </c>
-      <c r="B11" t="n">
+      <c r="C11" t="n">
         <v>9.210000000000001</v>
       </c>
-      <c r="C11" t="n">
+      <c r="D11" t="n">
         <v>11.05</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>2.99</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Gear_3_Ratio</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>9.039999999999999</v>
       </c>
-      <c r="B12" t="n">
+      <c r="C12" t="n">
         <v>7.09</v>
       </c>
-      <c r="C12" t="n">
+      <c r="D12" t="n">
         <v>8.41</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>2.15</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Gear_4_Ratio</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>7.09</v>
       </c>
-      <c r="B13" t="n">
+      <c r="C13" t="n">
         <v>5.57</v>
       </c>
-      <c r="C13" t="n">
+      <c r="D13" t="n">
         <v>6.43</v>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>1.8</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Gear_5_Ratio</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
         <v>5.54</v>
       </c>
-      <c r="B14" t="n">
+      <c r="C14" t="n">
         <v>4.35</v>
       </c>
-      <c r="C14" t="n">
+      <c r="D14" t="n">
         <v>4.95</v>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
         <v>1.52</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Gear_6_Ratio</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
         <v>4.35</v>
       </c>
-      <c r="B15" t="n">
+      <c r="C15" t="n">
         <v>3.41</v>
       </c>
-      <c r="C15" t="n">
+      <c r="D15" t="n">
         <v>3.79</v>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="n">
         <v>1.28</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Gear_7_Ratio</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
         <v>3.44</v>
       </c>
-      <c r="B16" t="n">
+      <c r="C16" t="n">
         <v>2.7</v>
       </c>
-      <c r="C16" t="n">
+      <c r="D16" t="n">
         <v>2.91</v>
       </c>
-      <c r="D16" t="n">
+      <c r="E16" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Gear_8_Ratio</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
         <v>2.7</v>
       </c>
-      <c r="B17" t="n">
+      <c r="C17" t="n">
         <v>2.12</v>
       </c>
-      <c r="C17" t="n">
+      <c r="D17" t="n">
         <v>2.23</v>
       </c>
-      <c r="D17" t="n">
+      <c r="E17" t="n">
         <v>0.85</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Gear_9_Ratio</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
         <v>2.08</v>
       </c>
-      <c r="B18" t="n">
+      <c r="C18" t="n">
         <v>1.63</v>
       </c>
-      <c r="C18" t="n">
+      <c r="D18" t="n">
         <v>1.7</v>
       </c>
-      <c r="D18" t="n">
+      <c r="E18" t="n">
         <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Gear_10_Ratio</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
         <v>1.63</v>
       </c>
-      <c r="B19" t="n">
+      <c r="C19" t="n">
         <v>1.28</v>
       </c>
-      <c r="C19" t="n">
+      <c r="D19" t="n">
         <v>1.3</v>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="n">
         <v>0.64</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Gear_11_Ratio</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
         <v>1.28</v>
-      </c>
-      <c r="B20" t="n">
-        <v>1</v>
       </c>
       <c r="C20" t="n">
         <v>1</v>
       </c>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Gear_12_Ratio</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
         <v>1</v>
       </c>
-      <c r="B21" t="n">
+      <c r="C21" t="n">
         <v>0.78</v>
       </c>
-      <c r="C21" t="n">
+      <c r="D21" t="n">
         <v>0.77</v>
       </c>
-      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>